<commit_message>
repeated api calls fixed
</commit_message>
<xml_diff>
--- a/electron/data/portfolio2.xlsx
+++ b/electron/data/portfolio2.xlsx
@@ -435,10 +435,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-10-01</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B3" t="str">
-        <v>hbl</v>
+        <v>EFERT</v>
       </c>
       <c r="C3" t="str">
         <v>Buy</v>
@@ -447,7 +447,7 @@
         <v>100</v>
       </c>
       <c r="E3" t="str">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
few bugs removed from dahsboard
</commit_message>
<xml_diff>
--- a/electron/data/portfolio2.xlsx
+++ b/electron/data/portfolio2.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -450,9 +450,26 @@
         <v>200</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2025-10-07</v>
+      </c>
+      <c r="B4" t="str">
+        <v>pael</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Buy</v>
+      </c>
+      <c r="D4" t="str">
+        <v>11</v>
+      </c>
+      <c r="E4" t="str">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>